<commit_message>
feat: implement M2E coefficient calculation and update related methods
</commit_message>
<xml_diff>
--- a/public/modeles/Annexe_MCCC.xlsx
+++ b/public/modeles/Annexe_MCCC.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10916"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10308"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/davidannebicque/Sites/oreof/public/modeles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F5006EE-A3F6-1B40-B7C3-2DEA36A2222D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8611444-E68C-6141-B40B-E1176AF9C14A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="35720" yWindow="1840" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="modele" sheetId="9" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="68">
   <si>
     <t>ACCREDITATION 2024-2028</t>
   </si>
@@ -52,15 +52,9 @@
     <t>Type de formation :</t>
   </si>
   <si>
-    <t>Licence</t>
-  </si>
-  <si>
     <t>Intitulé de la mention (Spécialité pour les BUT) :</t>
   </si>
   <si>
-    <t>LLCER</t>
-  </si>
-  <si>
     <t>Régime d'inscription :</t>
   </si>
   <si>
@@ -70,34 +64,19 @@
     <t>Intitulé du parcours (si existant) :</t>
   </si>
   <si>
-    <t>Anglais</t>
-  </si>
-  <si>
     <t>Formation continue</t>
   </si>
   <si>
-    <t>Année d'études :</t>
-  </si>
-  <si>
-    <t>1ère année</t>
-  </si>
-  <si>
     <t>Formation initiale en apprentissage</t>
   </si>
   <si>
     <t>Composante :</t>
   </si>
   <si>
-    <t>UFR Lettres et sciences humaines</t>
-  </si>
-  <si>
     <t>Formation continue en contrat de professionnalisation</t>
   </si>
   <si>
     <t>Site de formation :</t>
-  </si>
-  <si>
-    <t>Troyes</t>
   </si>
   <si>
     <t>Semestre</t>
@@ -1040,7 +1019,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="132">
+  <cellXfs count="130">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1273,32 +1252,62 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1351,83 +1360,47 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1924,38 +1897,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:36" ht="20" x14ac:dyDescent="0.2">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="84" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
-      <c r="AB1" s="117"/>
-      <c r="AC1" s="117"/>
-      <c r="AD1" s="117"/>
+      <c r="B1" s="84"/>
+      <c r="C1" s="84"/>
+      <c r="D1" s="84"/>
+      <c r="E1" s="84"/>
+      <c r="F1" s="84"/>
+      <c r="G1" s="84"/>
+      <c r="H1" s="84"/>
+      <c r="I1" s="84"/>
+      <c r="J1" s="84"/>
+      <c r="K1" s="84"/>
+      <c r="L1" s="84"/>
+      <c r="M1" s="84"/>
+      <c r="N1" s="84"/>
+      <c r="O1" s="84"/>
+      <c r="P1" s="84"/>
+      <c r="Q1" s="84"/>
+      <c r="R1" s="84"/>
+      <c r="S1" s="84"/>
+      <c r="T1" s="84"/>
+      <c r="U1" s="84"/>
+      <c r="V1" s="84"/>
+      <c r="W1" s="84"/>
+      <c r="X1" s="84"/>
+      <c r="Y1" s="84"/>
+      <c r="Z1" s="84"/>
+      <c r="AA1" s="84"/>
+      <c r="AB1" s="84"/>
+      <c r="AC1" s="84"/>
+      <c r="AD1" s="84"/>
       <c r="AE1" s="1"/>
       <c r="AF1" s="1"/>
       <c r="AG1" s="1"/>
@@ -1964,120 +1937,82 @@
       <c r="AJ1" s="1"/>
     </row>
     <row r="2" spans="1:36" ht="18" x14ac:dyDescent="0.2">
-      <c r="A2" s="118" t="s">
+      <c r="A2" s="85" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="118"/>
-      <c r="C2" s="118"/>
-      <c r="D2" s="118"/>
-      <c r="E2" s="118"/>
-      <c r="F2" s="118"/>
-      <c r="G2" s="118"/>
-      <c r="H2" s="118"/>
-      <c r="I2" s="118"/>
-      <c r="J2" s="118"/>
-      <c r="K2" s="118"/>
-      <c r="L2" s="118"/>
-      <c r="M2" s="118"/>
-      <c r="N2" s="118"/>
-      <c r="O2" s="118"/>
-      <c r="P2" s="118"/>
-      <c r="Q2" s="118"/>
-      <c r="R2" s="118"/>
-      <c r="S2" s="118"/>
-      <c r="T2" s="118"/>
-      <c r="U2" s="118"/>
-      <c r="V2" s="118"/>
-      <c r="W2" s="118"/>
-      <c r="X2" s="118"/>
-      <c r="Y2" s="118"/>
-      <c r="Z2" s="118"/>
-      <c r="AA2" s="118"/>
-      <c r="AB2" s="118"/>
-      <c r="AC2" s="118"/>
-      <c r="AD2" s="118"/>
+      <c r="B2" s="85"/>
+      <c r="C2" s="85"/>
+      <c r="D2" s="85"/>
+      <c r="E2" s="85"/>
+      <c r="F2" s="85"/>
+      <c r="G2" s="85"/>
+      <c r="H2" s="85"/>
+      <c r="I2" s="85"/>
+      <c r="J2" s="85"/>
+      <c r="K2" s="85"/>
+      <c r="L2" s="85"/>
+      <c r="M2" s="85"/>
+      <c r="N2" s="85"/>
+      <c r="O2" s="85"/>
+      <c r="P2" s="85"/>
+      <c r="Q2" s="85"/>
+      <c r="R2" s="85"/>
+      <c r="S2" s="85"/>
+      <c r="T2" s="85"/>
+      <c r="U2" s="85"/>
+      <c r="V2" s="85"/>
+      <c r="W2" s="85"/>
+      <c r="X2" s="85"/>
+      <c r="Y2" s="85"/>
+      <c r="Z2" s="85"/>
+      <c r="AA2" s="85"/>
+      <c r="AB2" s="85"/>
+      <c r="AC2" s="85"/>
+      <c r="AD2" s="85"/>
     </row>
     <row r="3" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="118" t="s">
+      <c r="A3" s="85" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="118"/>
-      <c r="C3" s="118"/>
-      <c r="D3" s="118"/>
-      <c r="E3" s="118"/>
-      <c r="F3" s="118"/>
-      <c r="G3" s="118"/>
-      <c r="H3" s="118"/>
-      <c r="I3" s="118"/>
-      <c r="J3" s="118"/>
-      <c r="K3" s="118"/>
-      <c r="L3" s="118"/>
-      <c r="M3" s="118"/>
-      <c r="N3" s="118"/>
-      <c r="O3" s="118"/>
-      <c r="P3" s="118"/>
-      <c r="Q3" s="118"/>
-      <c r="R3" s="118"/>
-      <c r="S3" s="118"/>
-      <c r="T3" s="118"/>
-      <c r="U3" s="118"/>
-      <c r="V3" s="118"/>
-      <c r="W3" s="118"/>
-      <c r="X3" s="118"/>
-      <c r="Y3" s="118"/>
-      <c r="Z3" s="118"/>
-      <c r="AA3" s="118"/>
-      <c r="AB3" s="118"/>
-      <c r="AC3" s="118"/>
-      <c r="AD3" s="118"/>
+      <c r="B3" s="85"/>
+      <c r="C3" s="85"/>
+      <c r="D3" s="85"/>
+      <c r="E3" s="85"/>
+      <c r="F3" s="85"/>
+      <c r="G3" s="85"/>
+      <c r="H3" s="85"/>
+      <c r="I3" s="85"/>
+      <c r="J3" s="85"/>
+      <c r="K3" s="85"/>
+      <c r="L3" s="85"/>
+      <c r="M3" s="85"/>
+      <c r="N3" s="85"/>
+      <c r="O3" s="85"/>
+      <c r="P3" s="85"/>
+      <c r="Q3" s="85"/>
+      <c r="R3" s="85"/>
+      <c r="S3" s="85"/>
+      <c r="T3" s="85"/>
+      <c r="U3" s="85"/>
+      <c r="V3" s="85"/>
+      <c r="W3" s="85"/>
+      <c r="X3" s="85"/>
+      <c r="Y3" s="85"/>
+      <c r="Z3" s="85"/>
+      <c r="AA3" s="85"/>
+      <c r="AB3" s="85"/>
+      <c r="AC3" s="85"/>
+      <c r="AD3" s="85"/>
     </row>
     <row r="4" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="G4" s="1"/>
     </row>
-    <row r="5" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="G5" s="88" t="s">
-        <v>3</v>
-      </c>
-      <c r="H5" s="88"/>
-      <c r="I5" s="88"/>
-      <c r="J5" s="112" t="s">
-        <v>4</v>
-      </c>
-      <c r="K5" s="112"/>
-      <c r="L5" s="112"/>
-      <c r="M5" s="1"/>
-      <c r="N5" s="1"/>
-      <c r="O5" s="1"/>
-      <c r="P5" s="1"/>
-      <c r="R5" s="1"/>
-      <c r="S5" s="1"/>
-      <c r="T5" s="1"/>
-    </row>
+    <row r="5" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="6" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C6" s="15"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
-      <c r="G6" s="88" t="s">
-        <v>5</v>
-      </c>
-      <c r="H6" s="88"/>
-      <c r="I6" s="88"/>
-      <c r="J6" s="112" t="s">
-        <v>6</v>
-      </c>
-      <c r="K6" s="112"/>
-      <c r="L6" s="112"/>
-      <c r="M6" s="112"/>
-      <c r="N6" s="112"/>
-      <c r="O6" s="112"/>
-      <c r="P6" s="112"/>
-      <c r="Q6" s="112"/>
-      <c r="R6" s="112"/>
-      <c r="S6" s="112"/>
-      <c r="T6" s="112"/>
-      <c r="U6" s="112"/>
-      <c r="V6" s="112"/>
       <c r="W6" s="2"/>
       <c r="X6" s="2"/>
       <c r="Y6" s="2"/>
@@ -2086,54 +2021,18 @@
     <row r="7" spans="1:36" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="7"/>
       <c r="C7" s="35" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D7" s="5"/>
       <c r="E7" s="37" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F7" s="7"/>
-      <c r="G7" s="88" t="s">
-        <v>9</v>
-      </c>
-      <c r="H7" s="88"/>
-      <c r="I7" s="88"/>
-      <c r="J7" s="112" t="s">
-        <v>10</v>
-      </c>
-      <c r="K7" s="112"/>
-      <c r="L7" s="112"/>
-      <c r="M7" s="112"/>
-      <c r="N7" s="112"/>
-      <c r="O7" s="112"/>
-      <c r="P7" s="112"/>
-      <c r="Q7" s="112"/>
-      <c r="R7" s="112"/>
-      <c r="S7" s="112"/>
-      <c r="T7" s="112"/>
-      <c r="U7" s="112"/>
-      <c r="V7" s="112"/>
     </row>
     <row r="8" spans="1:36" ht="5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D8" s="7"/>
       <c r="E8" s="6"/>
       <c r="F8" s="30"/>
-      <c r="G8" s="17"/>
-      <c r="H8" s="17"/>
-      <c r="I8" s="33"/>
-      <c r="J8" s="6"/>
-      <c r="K8" s="2"/>
-      <c r="L8" s="2"/>
-      <c r="M8" s="2"/>
-      <c r="N8" s="2"/>
-      <c r="O8" s="2"/>
-      <c r="P8" s="2"/>
-      <c r="Q8" s="2"/>
-      <c r="R8" s="2"/>
-      <c r="S8" s="2"/>
-      <c r="T8" s="2"/>
-      <c r="U8" s="2"/>
-      <c r="V8" s="2"/>
       <c r="W8" s="2"/>
       <c r="X8" s="2"/>
       <c r="Y8" s="2"/>
@@ -2144,29 +2043,9 @@
       <c r="A9" s="9"/>
       <c r="D9" s="5"/>
       <c r="E9" s="37" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F9" s="7"/>
-      <c r="G9" s="88" t="s">
-        <v>12</v>
-      </c>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="112" t="s">
-        <v>13</v>
-      </c>
-      <c r="K9" s="112"/>
-      <c r="L9" s="112"/>
-      <c r="M9" s="2"/>
-      <c r="N9" s="2"/>
-      <c r="O9" s="2"/>
-      <c r="P9" s="2"/>
-      <c r="Q9" s="3"/>
-      <c r="R9" s="2"/>
-      <c r="S9" s="2"/>
-      <c r="T9" s="2"/>
-      <c r="U9" s="3"/>
-      <c r="V9" s="3"/>
       <c r="W9" s="3"/>
       <c r="X9" s="3"/>
       <c r="Y9" s="3"/>
@@ -2176,61 +2055,25 @@
       <c r="D10" s="8"/>
       <c r="E10" s="32"/>
       <c r="F10" s="30"/>
-      <c r="G10" s="17"/>
-      <c r="H10" s="17"/>
-      <c r="I10" s="17"/>
-      <c r="J10" s="30"/>
-      <c r="K10" s="31"/>
-      <c r="L10" s="30"/>
-      <c r="M10" s="13"/>
     </row>
     <row r="11" spans="1:36" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D11" s="5"/>
       <c r="E11" s="37" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F11" s="7"/>
-      <c r="G11" s="88" t="s">
-        <v>15</v>
-      </c>
-      <c r="H11" s="88"/>
-      <c r="I11" s="88"/>
-      <c r="J11" s="112" t="s">
-        <v>16</v>
-      </c>
-      <c r="K11" s="112"/>
-      <c r="L11" s="112"/>
-      <c r="M11" s="12"/>
     </row>
     <row r="12" spans="1:36" ht="5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D12" s="6"/>
       <c r="E12" s="6"/>
       <c r="F12" s="30"/>
-      <c r="G12" s="17"/>
-      <c r="H12" s="17"/>
-      <c r="I12" s="17"/>
-      <c r="J12" s="32"/>
-      <c r="K12" s="12"/>
-      <c r="L12" s="30"/>
-      <c r="M12" s="12"/>
     </row>
     <row r="13" spans="1:36" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D13" s="5"/>
       <c r="E13" s="37" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="F13" s="7"/>
-      <c r="G13" s="88" t="s">
-        <v>18</v>
-      </c>
-      <c r="H13" s="88"/>
-      <c r="I13" s="88"/>
-      <c r="J13" s="112" t="s">
-        <v>19</v>
-      </c>
-      <c r="K13" s="112"/>
-      <c r="L13" s="112"/>
-      <c r="M13" s="12"/>
     </row>
     <row r="14" spans="1:36" ht="8" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="C14"/>
@@ -2240,180 +2083,180 @@
       <c r="M14"/>
     </row>
     <row r="15" spans="1:36" s="39" customFormat="1" ht="19.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="92" t="s">
+      <c r="A15" s="102" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" s="105" t="s">
+        <v>14</v>
+      </c>
+      <c r="C15" s="106"/>
+      <c r="D15" s="94" t="s">
+        <v>15</v>
+      </c>
+      <c r="E15" s="94"/>
+      <c r="F15" s="94"/>
+      <c r="G15" s="94"/>
+      <c r="H15" s="94"/>
+      <c r="I15" s="94"/>
+      <c r="J15" s="94"/>
+      <c r="K15" s="94"/>
+      <c r="L15" s="94"/>
+      <c r="M15" s="95"/>
+      <c r="N15" s="98" t="s">
+        <v>16</v>
+      </c>
+      <c r="O15" s="91"/>
+      <c r="P15" s="91"/>
+      <c r="Q15" s="91"/>
+      <c r="R15" s="91"/>
+      <c r="S15" s="91"/>
+      <c r="T15" s="91"/>
+      <c r="U15" s="91"/>
+      <c r="V15" s="91"/>
+      <c r="W15" s="92"/>
+      <c r="X15" s="91" t="s">
+        <v>17</v>
+      </c>
+      <c r="Y15" s="91"/>
+      <c r="Z15" s="92"/>
+      <c r="AA15" s="120" t="s">
+        <v>47</v>
+      </c>
+      <c r="AB15" s="120"/>
+      <c r="AC15" s="120"/>
+      <c r="AD15" s="121"/>
+    </row>
+    <row r="16" spans="1:36" s="39" customFormat="1" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="103"/>
+      <c r="B16" s="107"/>
+      <c r="C16" s="108"/>
+      <c r="D16" s="96"/>
+      <c r="E16" s="96"/>
+      <c r="F16" s="96"/>
+      <c r="G16" s="96"/>
+      <c r="H16" s="96"/>
+      <c r="I16" s="96"/>
+      <c r="J16" s="96"/>
+      <c r="K16" s="96"/>
+      <c r="L16" s="96"/>
+      <c r="M16" s="97"/>
+      <c r="N16" s="98" t="s">
+        <v>18</v>
+      </c>
+      <c r="O16" s="91"/>
+      <c r="P16" s="91"/>
+      <c r="Q16" s="118"/>
+      <c r="R16" s="98" t="s">
+        <v>19</v>
+      </c>
+      <c r="S16" s="91"/>
+      <c r="T16" s="91"/>
+      <c r="U16" s="118"/>
+      <c r="V16" s="116" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="95" t="s">
+      <c r="W16" s="109" t="s">
+        <v>55</v>
+      </c>
+      <c r="X16" s="87" t="s">
+        <v>49</v>
+      </c>
+      <c r="Y16" s="89" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z16" s="126" t="s">
+        <v>46</v>
+      </c>
+      <c r="AA16" s="122" t="s">
+        <v>54</v>
+      </c>
+      <c r="AB16" s="123"/>
+      <c r="AC16" s="124" t="s">
+        <v>50</v>
+      </c>
+      <c r="AD16" s="124" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="17" spans="1:30" s="44" customFormat="1" ht="44" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="104"/>
+      <c r="B17" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="C15" s="96"/>
-      <c r="D15" s="125" t="s">
+      <c r="C17" s="40" t="s">
+        <v>48</v>
+      </c>
+      <c r="D17" s="41" t="s">
         <v>22</v>
       </c>
-      <c r="E15" s="125"/>
-      <c r="F15" s="125"/>
-      <c r="G15" s="125"/>
-      <c r="H15" s="125"/>
-      <c r="I15" s="125"/>
-      <c r="J15" s="125"/>
-      <c r="K15" s="125"/>
-      <c r="L15" s="125"/>
-      <c r="M15" s="126"/>
-      <c r="N15" s="109" t="s">
+      <c r="E17" s="40" t="s">
         <v>23</v>
       </c>
-      <c r="O15" s="110"/>
-      <c r="P15" s="110"/>
-      <c r="Q15" s="110"/>
-      <c r="R15" s="110"/>
-      <c r="S15" s="110"/>
-      <c r="T15" s="110"/>
-      <c r="U15" s="110"/>
-      <c r="V15" s="110"/>
-      <c r="W15" s="123"/>
-      <c r="X15" s="110" t="s">
+      <c r="F17" s="40" t="s">
         <v>24</v>
       </c>
-      <c r="Y15" s="110"/>
-      <c r="Z15" s="123"/>
-      <c r="AA15" s="80" t="s">
-        <v>54</v>
-      </c>
-      <c r="AB15" s="80"/>
-      <c r="AC15" s="80"/>
-      <c r="AD15" s="81"/>
-    </row>
-    <row r="16" spans="1:36" s="39" customFormat="1" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="93"/>
-      <c r="B16" s="97"/>
-      <c r="C16" s="98"/>
-      <c r="D16" s="127"/>
-      <c r="E16" s="127"/>
-      <c r="F16" s="127"/>
-      <c r="G16" s="127"/>
-      <c r="H16" s="127"/>
-      <c r="I16" s="127"/>
-      <c r="J16" s="127"/>
-      <c r="K16" s="127"/>
-      <c r="L16" s="127"/>
-      <c r="M16" s="128"/>
-      <c r="N16" s="109" t="s">
+      <c r="G17" s="42" t="s">
         <v>25</v>
       </c>
-      <c r="O16" s="110"/>
-      <c r="P16" s="110"/>
-      <c r="Q16" s="111"/>
-      <c r="R16" s="109" t="s">
+      <c r="H17" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="S16" s="110"/>
-      <c r="T16" s="110"/>
-      <c r="U16" s="111"/>
-      <c r="V16" s="107" t="s">
+      <c r="I17" s="42" t="s">
         <v>27</v>
       </c>
-      <c r="W16" s="99" t="s">
-        <v>62</v>
-      </c>
-      <c r="X16" s="119" t="s">
-        <v>56</v>
-      </c>
-      <c r="Y16" s="121" t="s">
+      <c r="J17" s="42" t="s">
+        <v>28</v>
+      </c>
+      <c r="K17" s="42" t="s">
+        <v>65</v>
+      </c>
+      <c r="L17" s="42" t="s">
+        <v>41</v>
+      </c>
+      <c r="M17" s="43" t="s">
+        <v>29</v>
+      </c>
+      <c r="N17" s="54" t="s">
+        <v>30</v>
+      </c>
+      <c r="O17" s="55" t="s">
+        <v>31</v>
+      </c>
+      <c r="P17" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q17" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="R17" s="48" t="s">
+        <v>30</v>
+      </c>
+      <c r="S17" s="55" t="s">
+        <v>31</v>
+      </c>
+      <c r="T17" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="U17" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="V17" s="117"/>
+      <c r="W17" s="110"/>
+      <c r="X17" s="88"/>
+      <c r="Y17" s="90"/>
+      <c r="Z17" s="127"/>
+      <c r="AA17" s="49" t="s">
         <v>52</v>
       </c>
-      <c r="Z16" s="86" t="s">
+      <c r="AB17" s="38" t="s">
         <v>53</v>
       </c>
-      <c r="AA16" s="82" t="s">
-        <v>61</v>
-      </c>
-      <c r="AB16" s="83"/>
-      <c r="AC16" s="84" t="s">
-        <v>57</v>
-      </c>
-      <c r="AD16" s="84" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="17" spans="1:30" s="44" customFormat="1" ht="44" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="94"/>
-      <c r="B17" s="41" t="s">
-        <v>28</v>
-      </c>
-      <c r="C17" s="40" t="s">
-        <v>55</v>
-      </c>
-      <c r="D17" s="41" t="s">
-        <v>29</v>
-      </c>
-      <c r="E17" s="40" t="s">
-        <v>30</v>
-      </c>
-      <c r="F17" s="40" t="s">
-        <v>31</v>
-      </c>
-      <c r="G17" s="42" t="s">
-        <v>32</v>
-      </c>
-      <c r="H17" s="42" t="s">
-        <v>33</v>
-      </c>
-      <c r="I17" s="42" t="s">
-        <v>34</v>
-      </c>
-      <c r="J17" s="42" t="s">
-        <v>35</v>
-      </c>
-      <c r="K17" s="42" t="s">
-        <v>72</v>
-      </c>
-      <c r="L17" s="42" t="s">
-        <v>48</v>
-      </c>
-      <c r="M17" s="43" t="s">
-        <v>36</v>
-      </c>
-      <c r="N17" s="54" t="s">
-        <v>37</v>
-      </c>
-      <c r="O17" s="55" t="s">
-        <v>38</v>
-      </c>
-      <c r="P17" s="14" t="s">
-        <v>39</v>
-      </c>
-      <c r="Q17" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="R17" s="48" t="s">
-        <v>37</v>
-      </c>
-      <c r="S17" s="55" t="s">
-        <v>38</v>
-      </c>
-      <c r="T17" s="14" t="s">
-        <v>39</v>
-      </c>
-      <c r="U17" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="V17" s="108"/>
-      <c r="W17" s="100"/>
-      <c r="X17" s="120"/>
-      <c r="Y17" s="122"/>
-      <c r="Z17" s="87"/>
-      <c r="AA17" s="49" t="s">
-        <v>59</v>
-      </c>
-      <c r="AB17" s="38" t="s">
-        <v>60</v>
-      </c>
-      <c r="AC17" s="85"/>
-      <c r="AD17" s="85"/>
+      <c r="AC17" s="125"/>
+      <c r="AD17" s="125"/>
     </row>
     <row r="18" spans="1:30" ht="44" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A18" s="18" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="B18" s="19">
         <v>11</v>
@@ -2450,19 +2293,19 @@
       <c r="AD18" s="47"/>
     </row>
     <row r="19" spans="1:30" ht="44" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="124" t="s">
-        <v>73</v>
-      </c>
-      <c r="B19" s="124"/>
-      <c r="C19" s="124"/>
-      <c r="D19" s="124"/>
-      <c r="E19" s="124"/>
+      <c r="A19" s="93" t="s">
+        <v>66</v>
+      </c>
+      <c r="B19" s="93"/>
+      <c r="C19" s="93"/>
+      <c r="D19" s="93"/>
+      <c r="E19" s="93"/>
       <c r="F19" s="36"/>
       <c r="H19" s="11"/>
-      <c r="L19" s="105" t="s">
-        <v>49</v>
-      </c>
-      <c r="M19" s="105"/>
+      <c r="L19" s="115" t="s">
+        <v>42</v>
+      </c>
+      <c r="M19" s="115"/>
       <c r="N19" s="64"/>
       <c r="O19" s="65"/>
       <c r="P19" s="66"/>
@@ -2482,69 +2325,69 @@
       <c r="AD19" s="47"/>
     </row>
     <row r="20" spans="1:30" ht="75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="101" t="s">
-        <v>63</v>
-      </c>
-      <c r="B20" s="101"/>
-      <c r="C20" s="101"/>
-      <c r="D20" s="101"/>
-      <c r="E20" s="101"/>
+      <c r="A20" s="111" t="s">
+        <v>56</v>
+      </c>
+      <c r="B20" s="111"/>
+      <c r="C20" s="111"/>
+      <c r="D20" s="111"/>
+      <c r="E20" s="111"/>
       <c r="H20" s="11"/>
-      <c r="L20" s="106" t="s">
-        <v>50</v>
-      </c>
-      <c r="M20" s="106"/>
-      <c r="N20" s="102"/>
-      <c r="O20" s="103"/>
-      <c r="P20" s="103"/>
-      <c r="Q20" s="103"/>
-      <c r="R20" s="103"/>
-      <c r="S20" s="103"/>
-      <c r="T20" s="103"/>
-      <c r="U20" s="103"/>
-      <c r="V20" s="104"/>
+      <c r="L20" s="86" t="s">
+        <v>43</v>
+      </c>
+      <c r="M20" s="86"/>
+      <c r="N20" s="112"/>
+      <c r="O20" s="113"/>
+      <c r="P20" s="113"/>
+      <c r="Q20" s="113"/>
+      <c r="R20" s="113"/>
+      <c r="S20" s="113"/>
+      <c r="T20" s="113"/>
+      <c r="U20" s="113"/>
+      <c r="V20" s="114"/>
       <c r="W20" s="67"/>
     </row>
     <row r="21" spans="1:30" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="131" t="s">
-        <v>74</v>
-      </c>
-      <c r="B21" s="131"/>
-      <c r="C21" s="131"/>
-      <c r="D21" s="131"/>
-      <c r="E21" s="131"/>
+      <c r="A21" s="119" t="s">
+        <v>67</v>
+      </c>
+      <c r="B21" s="119"/>
+      <c r="C21" s="119"/>
+      <c r="D21" s="119"/>
+      <c r="E21" s="119"/>
       <c r="H21" s="11"/>
-      <c r="L21" s="106" t="s">
-        <v>47</v>
-      </c>
-      <c r="M21" s="106"/>
-      <c r="N21" s="89"/>
-      <c r="O21" s="90"/>
-      <c r="P21" s="90"/>
-      <c r="Q21" s="90"/>
-      <c r="R21" s="90"/>
-      <c r="S21" s="90"/>
-      <c r="T21" s="90"/>
-      <c r="U21" s="90"/>
-      <c r="V21" s="90"/>
-      <c r="W21" s="91"/>
+      <c r="L21" s="86" t="s">
+        <v>40</v>
+      </c>
+      <c r="M21" s="86"/>
+      <c r="N21" s="99"/>
+      <c r="O21" s="100"/>
+      <c r="P21" s="100"/>
+      <c r="Q21" s="100"/>
+      <c r="R21" s="100"/>
+      <c r="S21" s="100"/>
+      <c r="T21" s="100"/>
+      <c r="U21" s="100"/>
+      <c r="V21" s="100"/>
+      <c r="W21" s="101"/>
     </row>
     <row r="22" spans="1:30" ht="31" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A22" s="4"/>
       <c r="H22" s="11"/>
-      <c r="L22" s="106" t="s">
-        <v>64</v>
-      </c>
-      <c r="M22" s="106"/>
-      <c r="N22" s="89"/>
-      <c r="O22" s="90"/>
-      <c r="P22" s="90"/>
-      <c r="Q22" s="90"/>
-      <c r="R22" s="90"/>
-      <c r="S22" s="90"/>
-      <c r="T22" s="90"/>
-      <c r="U22" s="90"/>
-      <c r="V22" s="91"/>
+      <c r="L22" s="86" t="s">
+        <v>57</v>
+      </c>
+      <c r="M22" s="86"/>
+      <c r="N22" s="99"/>
+      <c r="O22" s="100"/>
+      <c r="P22" s="100"/>
+      <c r="Q22" s="100"/>
+      <c r="R22" s="100"/>
+      <c r="S22" s="100"/>
+      <c r="T22" s="100"/>
+      <c r="U22" s="100"/>
+      <c r="V22" s="101"/>
       <c r="W22" s="67"/>
     </row>
     <row r="23" spans="1:30" ht="16" thickBot="1" x14ac:dyDescent="0.25">
@@ -2553,45 +2396,63 @@
     </row>
     <row r="24" spans="1:30" ht="34" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="C24" s="29" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="D24" s="58"/>
       <c r="E24" s="59"/>
       <c r="Z24" s="11"/>
       <c r="AA24" s="61" t="s">
-        <v>44</v>
-      </c>
-      <c r="AB24" s="114"/>
-      <c r="AC24" s="115"/>
-      <c r="AD24" s="116"/>
+        <v>37</v>
+      </c>
+      <c r="AB24" s="81"/>
+      <c r="AC24" s="82"/>
+      <c r="AD24" s="83"/>
     </row>
     <row r="25" spans="1:30" ht="34" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A25" s="11"/>
       <c r="B25" s="11"/>
       <c r="C25" s="61" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="D25" s="57"/>
       <c r="E25" s="60"/>
       <c r="Z25" s="56"/>
       <c r="AA25" s="61" t="s">
-        <v>46</v>
-      </c>
-      <c r="AB25" s="114"/>
-      <c r="AC25" s="115"/>
-      <c r="AD25" s="116"/>
+        <v>39</v>
+      </c>
+      <c r="AB25" s="81"/>
+      <c r="AC25" s="82"/>
+      <c r="AD25" s="83"/>
     </row>
     <row r="27" spans="1:30" ht="111" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="113" t="s">
-        <v>71</v>
-      </c>
-      <c r="B27" s="113"/>
-      <c r="C27" s="113"/>
-      <c r="D27" s="113"/>
-      <c r="E27" s="113"/>
+      <c r="A27" s="80" t="s">
+        <v>64</v>
+      </c>
+      <c r="B27" s="80"/>
+      <c r="C27" s="80"/>
+      <c r="D27" s="80"/>
+      <c r="E27" s="80"/>
     </row>
   </sheetData>
-  <mergeCells count="44">
+  <mergeCells count="32">
+    <mergeCell ref="AA15:AD15"/>
+    <mergeCell ref="AA16:AB16"/>
+    <mergeCell ref="AC16:AC17"/>
+    <mergeCell ref="AD16:AD17"/>
+    <mergeCell ref="Z16:Z17"/>
+    <mergeCell ref="N22:V22"/>
+    <mergeCell ref="A15:A17"/>
+    <mergeCell ref="B15:C16"/>
+    <mergeCell ref="W16:W17"/>
+    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="N20:V20"/>
+    <mergeCell ref="N21:W21"/>
+    <mergeCell ref="L19:M19"/>
+    <mergeCell ref="L20:M20"/>
+    <mergeCell ref="V16:V17"/>
+    <mergeCell ref="R16:U16"/>
+    <mergeCell ref="N16:Q16"/>
+    <mergeCell ref="A21:E21"/>
     <mergeCell ref="A27:E27"/>
     <mergeCell ref="AB25:AD25"/>
     <mergeCell ref="A1:AD1"/>
@@ -2604,38 +2465,8 @@
     <mergeCell ref="X15:Z15"/>
     <mergeCell ref="A19:E19"/>
     <mergeCell ref="L21:M21"/>
-    <mergeCell ref="G5:I5"/>
-    <mergeCell ref="J5:L5"/>
     <mergeCell ref="D15:M16"/>
     <mergeCell ref="N15:W15"/>
-    <mergeCell ref="G6:I6"/>
-    <mergeCell ref="G7:I7"/>
-    <mergeCell ref="G9:I9"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="J6:V6"/>
-    <mergeCell ref="J7:V7"/>
-    <mergeCell ref="J11:L11"/>
-    <mergeCell ref="J9:L9"/>
-    <mergeCell ref="G13:I13"/>
-    <mergeCell ref="N22:V22"/>
-    <mergeCell ref="A15:A17"/>
-    <mergeCell ref="B15:C16"/>
-    <mergeCell ref="W16:W17"/>
-    <mergeCell ref="A20:E20"/>
-    <mergeCell ref="N20:V20"/>
-    <mergeCell ref="N21:W21"/>
-    <mergeCell ref="L19:M19"/>
-    <mergeCell ref="L20:M20"/>
-    <mergeCell ref="V16:V17"/>
-    <mergeCell ref="R16:U16"/>
-    <mergeCell ref="N16:Q16"/>
-    <mergeCell ref="J13:L13"/>
-    <mergeCell ref="A21:E21"/>
-    <mergeCell ref="AA15:AD15"/>
-    <mergeCell ref="AA16:AB16"/>
-    <mergeCell ref="AC16:AC17"/>
-    <mergeCell ref="AD16:AD17"/>
-    <mergeCell ref="Z16:Z17"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -2663,15 +2494,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:53" ht="20" x14ac:dyDescent="0.2">
-      <c r="A1" s="129" t="s">
+      <c r="A1" s="128" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="129"/>
-      <c r="C1" s="129"/>
-      <c r="D1" s="129"/>
-      <c r="E1" s="129"/>
-      <c r="F1" s="129"/>
-      <c r="G1" s="129"/>
+      <c r="B1" s="128"/>
+      <c r="C1" s="128"/>
+      <c r="D1" s="128"/>
+      <c r="E1" s="128"/>
+      <c r="F1" s="128"/>
+      <c r="G1" s="128"/>
       <c r="H1" s="62"/>
       <c r="I1" s="62"/>
       <c r="J1" s="62"/>
@@ -2710,15 +2541,15 @@
       <c r="BA1" s="1"/>
     </row>
     <row r="2" spans="1:53" ht="18" x14ac:dyDescent="0.2">
-      <c r="A2" s="130" t="s">
-        <v>51</v>
-      </c>
-      <c r="B2" s="130"/>
-      <c r="C2" s="130"/>
-      <c r="D2" s="130"/>
-      <c r="E2" s="130"/>
-      <c r="F2" s="130"/>
-      <c r="G2" s="130"/>
+      <c r="A2" s="129" t="s">
+        <v>44</v>
+      </c>
+      <c r="B2" s="129"/>
+      <c r="C2" s="129"/>
+      <c r="D2" s="129"/>
+      <c r="E2" s="129"/>
+      <c r="F2" s="129"/>
+      <c r="G2" s="129"/>
       <c r="H2" s="63"/>
       <c r="I2" s="63"/>
       <c r="J2" s="63"/>
@@ -2739,15 +2570,15 @@
       <c r="Y2" s="63"/>
     </row>
     <row r="3" spans="1:53" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="130" t="s">
-        <v>65</v>
-      </c>
-      <c r="B3" s="130"/>
-      <c r="C3" s="130"/>
-      <c r="D3" s="130"/>
-      <c r="E3" s="130"/>
-      <c r="F3" s="130"/>
-      <c r="G3" s="130"/>
+      <c r="A3" s="129" t="s">
+        <v>58</v>
+      </c>
+      <c r="B3" s="129"/>
+      <c r="C3" s="129"/>
+      <c r="D3" s="129"/>
+      <c r="E3" s="129"/>
+      <c r="F3" s="129"/>
+      <c r="G3" s="129"/>
       <c r="H3" s="63"/>
       <c r="I3" s="63"/>
       <c r="J3" s="63"/>
@@ -2783,7 +2614,7 @@
         <v>3</v>
       </c>
       <c r="D5" s="78" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="E5" s="78"/>
       <c r="F5" s="78"/>
@@ -2805,10 +2636,10 @@
     <row r="6" spans="1:53" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="4"/>
       <c r="C6" s="71" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D6" s="78" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="E6" s="78"/>
       <c r="F6" s="78"/>
@@ -2847,10 +2678,10 @@
       <c r="A7" s="72"/>
       <c r="B7" s="4"/>
       <c r="C7" s="71" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D7" s="78" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="E7" s="78"/>
       <c r="F7" s="78"/>
@@ -2969,10 +2800,10 @@
     <row r="11" spans="1:53" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="4"/>
       <c r="C11" s="71" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D11" s="78" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="E11" s="78"/>
       <c r="F11" s="78"/>
@@ -3001,10 +2832,10 @@
     <row r="13" spans="1:53" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="4"/>
       <c r="C13" s="71" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="D13" s="78" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="E13" s="78"/>
       <c r="F13" s="78"/>
@@ -3029,15 +2860,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="026a8ae5-d6a9-4af7-bf98-fe61cc11d283" xsi:nil="true"/>
@@ -3046,6 +2868,15 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3266,20 +3097,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AD87B94F-381C-458D-A5C9-64DD7F51B7FF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DE9C2EEE-EA72-4039-9998-752A033046FC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="026a8ae5-d6a9-4af7-bf98-fe61cc11d283"/>
     <ds:schemaRef ds:uri="8103b6e4-b1cc-417b-af38-f980b3f4bdef"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AD87B94F-381C-458D-A5C9-64DD7F51B7FF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
feat: add co-responsable field and update formation handling in forms
</commit_message>
<xml_diff>
--- a/public/modeles/Annexe_MCCC.xlsx
+++ b/public/modeles/Annexe_MCCC.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/davidannebicque/Sites/oreof/public/modeles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8611444-E68C-6141-B40B-E1176AF9C14A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C34C18E3-214E-AD43-80CA-65C0E07D4B2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="35720" yWindow="1840" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="modele" sheetId="9" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="75">
   <si>
     <t>ACCREDITATION 2024-2028</t>
   </si>
@@ -246,6 +246,27 @@
   </si>
   <si>
     <t>*** Les choix d'EC dans le cas d'EC à choix restreint ou libre doivent être différent au sein d'un même semestre</t>
+  </si>
+  <si>
+    <t>Licence</t>
+  </si>
+  <si>
+    <t>LLCER</t>
+  </si>
+  <si>
+    <t>Anglais</t>
+  </si>
+  <si>
+    <t>Année d'études :</t>
+  </si>
+  <si>
+    <t>1ère année</t>
+  </si>
+  <si>
+    <t>UFR Lettres et sciences humaines</t>
+  </si>
+  <si>
+    <t>Troyes</t>
   </si>
 </sst>
 </file>
@@ -1019,7 +1040,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="130">
+  <cellXfs count="132">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1252,6 +1273,102 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1270,9 +1387,6 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1283,9 +1397,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1306,101 +1417,17 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1897,38 +1924,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:36" ht="20" x14ac:dyDescent="0.2">
-      <c r="A1" s="84" t="s">
+      <c r="A1" s="116" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="84"/>
-      <c r="C1" s="84"/>
-      <c r="D1" s="84"/>
-      <c r="E1" s="84"/>
-      <c r="F1" s="84"/>
-      <c r="G1" s="84"/>
-      <c r="H1" s="84"/>
-      <c r="I1" s="84"/>
-      <c r="J1" s="84"/>
-      <c r="K1" s="84"/>
-      <c r="L1" s="84"/>
-      <c r="M1" s="84"/>
-      <c r="N1" s="84"/>
-      <c r="O1" s="84"/>
-      <c r="P1" s="84"/>
-      <c r="Q1" s="84"/>
-      <c r="R1" s="84"/>
-      <c r="S1" s="84"/>
-      <c r="T1" s="84"/>
-      <c r="U1" s="84"/>
-      <c r="V1" s="84"/>
-      <c r="W1" s="84"/>
-      <c r="X1" s="84"/>
-      <c r="Y1" s="84"/>
-      <c r="Z1" s="84"/>
-      <c r="AA1" s="84"/>
-      <c r="AB1" s="84"/>
-      <c r="AC1" s="84"/>
-      <c r="AD1" s="84"/>
+      <c r="B1" s="116"/>
+      <c r="C1" s="116"/>
+      <c r="D1" s="116"/>
+      <c r="E1" s="116"/>
+      <c r="F1" s="116"/>
+      <c r="G1" s="116"/>
+      <c r="H1" s="116"/>
+      <c r="I1" s="116"/>
+      <c r="J1" s="116"/>
+      <c r="K1" s="116"/>
+      <c r="L1" s="116"/>
+      <c r="M1" s="116"/>
+      <c r="N1" s="116"/>
+      <c r="O1" s="116"/>
+      <c r="P1" s="116"/>
+      <c r="Q1" s="116"/>
+      <c r="R1" s="116"/>
+      <c r="S1" s="116"/>
+      <c r="T1" s="116"/>
+      <c r="U1" s="116"/>
+      <c r="V1" s="116"/>
+      <c r="W1" s="116"/>
+      <c r="X1" s="116"/>
+      <c r="Y1" s="116"/>
+      <c r="Z1" s="116"/>
+      <c r="AA1" s="116"/>
+      <c r="AB1" s="116"/>
+      <c r="AC1" s="116"/>
+      <c r="AD1" s="116"/>
       <c r="AE1" s="1"/>
       <c r="AF1" s="1"/>
       <c r="AG1" s="1"/>
@@ -1937,82 +1964,120 @@
       <c r="AJ1" s="1"/>
     </row>
     <row r="2" spans="1:36" ht="18" x14ac:dyDescent="0.2">
-      <c r="A2" s="85" t="s">
+      <c r="A2" s="117" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="85"/>
-      <c r="C2" s="85"/>
-      <c r="D2" s="85"/>
-      <c r="E2" s="85"/>
-      <c r="F2" s="85"/>
-      <c r="G2" s="85"/>
-      <c r="H2" s="85"/>
-      <c r="I2" s="85"/>
-      <c r="J2" s="85"/>
-      <c r="K2" s="85"/>
-      <c r="L2" s="85"/>
-      <c r="M2" s="85"/>
-      <c r="N2" s="85"/>
-      <c r="O2" s="85"/>
-      <c r="P2" s="85"/>
-      <c r="Q2" s="85"/>
-      <c r="R2" s="85"/>
-      <c r="S2" s="85"/>
-      <c r="T2" s="85"/>
-      <c r="U2" s="85"/>
-      <c r="V2" s="85"/>
-      <c r="W2" s="85"/>
-      <c r="X2" s="85"/>
-      <c r="Y2" s="85"/>
-      <c r="Z2" s="85"/>
-      <c r="AA2" s="85"/>
-      <c r="AB2" s="85"/>
-      <c r="AC2" s="85"/>
-      <c r="AD2" s="85"/>
+      <c r="B2" s="117"/>
+      <c r="C2" s="117"/>
+      <c r="D2" s="117"/>
+      <c r="E2" s="117"/>
+      <c r="F2" s="117"/>
+      <c r="G2" s="117"/>
+      <c r="H2" s="117"/>
+      <c r="I2" s="117"/>
+      <c r="J2" s="117"/>
+      <c r="K2" s="117"/>
+      <c r="L2" s="117"/>
+      <c r="M2" s="117"/>
+      <c r="N2" s="117"/>
+      <c r="O2" s="117"/>
+      <c r="P2" s="117"/>
+      <c r="Q2" s="117"/>
+      <c r="R2" s="117"/>
+      <c r="S2" s="117"/>
+      <c r="T2" s="117"/>
+      <c r="U2" s="117"/>
+      <c r="V2" s="117"/>
+      <c r="W2" s="117"/>
+      <c r="X2" s="117"/>
+      <c r="Y2" s="117"/>
+      <c r="Z2" s="117"/>
+      <c r="AA2" s="117"/>
+      <c r="AB2" s="117"/>
+      <c r="AC2" s="117"/>
+      <c r="AD2" s="117"/>
     </row>
     <row r="3" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="85" t="s">
+      <c r="A3" s="117" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="85"/>
-      <c r="C3" s="85"/>
-      <c r="D3" s="85"/>
-      <c r="E3" s="85"/>
-      <c r="F3" s="85"/>
-      <c r="G3" s="85"/>
-      <c r="H3" s="85"/>
-      <c r="I3" s="85"/>
-      <c r="J3" s="85"/>
-      <c r="K3" s="85"/>
-      <c r="L3" s="85"/>
-      <c r="M3" s="85"/>
-      <c r="N3" s="85"/>
-      <c r="O3" s="85"/>
-      <c r="P3" s="85"/>
-      <c r="Q3" s="85"/>
-      <c r="R3" s="85"/>
-      <c r="S3" s="85"/>
-      <c r="T3" s="85"/>
-      <c r="U3" s="85"/>
-      <c r="V3" s="85"/>
-      <c r="W3" s="85"/>
-      <c r="X3" s="85"/>
-      <c r="Y3" s="85"/>
-      <c r="Z3" s="85"/>
-      <c r="AA3" s="85"/>
-      <c r="AB3" s="85"/>
-      <c r="AC3" s="85"/>
-      <c r="AD3" s="85"/>
+      <c r="B3" s="117"/>
+      <c r="C3" s="117"/>
+      <c r="D3" s="117"/>
+      <c r="E3" s="117"/>
+      <c r="F3" s="117"/>
+      <c r="G3" s="117"/>
+      <c r="H3" s="117"/>
+      <c r="I3" s="117"/>
+      <c r="J3" s="117"/>
+      <c r="K3" s="117"/>
+      <c r="L3" s="117"/>
+      <c r="M3" s="117"/>
+      <c r="N3" s="117"/>
+      <c r="O3" s="117"/>
+      <c r="P3" s="117"/>
+      <c r="Q3" s="117"/>
+      <c r="R3" s="117"/>
+      <c r="S3" s="117"/>
+      <c r="T3" s="117"/>
+      <c r="U3" s="117"/>
+      <c r="V3" s="117"/>
+      <c r="W3" s="117"/>
+      <c r="X3" s="117"/>
+      <c r="Y3" s="117"/>
+      <c r="Z3" s="117"/>
+      <c r="AA3" s="117"/>
+      <c r="AB3" s="117"/>
+      <c r="AC3" s="117"/>
+      <c r="AD3" s="117"/>
     </row>
     <row r="4" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="G4" s="1"/>
     </row>
-    <row r="5" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="5" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G5" s="130" t="s">
+        <v>3</v>
+      </c>
+      <c r="H5" s="130"/>
+      <c r="I5" s="130"/>
+      <c r="J5" s="131" t="s">
+        <v>68</v>
+      </c>
+      <c r="K5" s="131"/>
+      <c r="L5" s="131"/>
+      <c r="M5" s="1"/>
+      <c r="N5" s="1"/>
+      <c r="O5" s="1"/>
+      <c r="P5" s="1"/>
+      <c r="R5" s="1"/>
+      <c r="S5" s="1"/>
+      <c r="T5" s="1"/>
+    </row>
     <row r="6" spans="1:36" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C6" s="15"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
+      <c r="G6" s="130" t="s">
+        <v>4</v>
+      </c>
+      <c r="H6" s="130"/>
+      <c r="I6" s="130"/>
+      <c r="J6" s="131" t="s">
+        <v>69</v>
+      </c>
+      <c r="K6" s="131"/>
+      <c r="L6" s="131"/>
+      <c r="M6" s="131"/>
+      <c r="N6" s="131"/>
+      <c r="O6" s="131"/>
+      <c r="P6" s="131"/>
+      <c r="Q6" s="131"/>
+      <c r="R6" s="131"/>
+      <c r="S6" s="131"/>
+      <c r="T6" s="131"/>
+      <c r="U6" s="131"/>
+      <c r="V6" s="131"/>
       <c r="W6" s="2"/>
       <c r="X6" s="2"/>
       <c r="Y6" s="2"/>
@@ -2028,11 +2093,47 @@
         <v>6</v>
       </c>
       <c r="F7" s="7"/>
+      <c r="G7" s="130" t="s">
+        <v>7</v>
+      </c>
+      <c r="H7" s="130"/>
+      <c r="I7" s="130"/>
+      <c r="J7" s="131" t="s">
+        <v>70</v>
+      </c>
+      <c r="K7" s="131"/>
+      <c r="L7" s="131"/>
+      <c r="M7" s="131"/>
+      <c r="N7" s="131"/>
+      <c r="O7" s="131"/>
+      <c r="P7" s="131"/>
+      <c r="Q7" s="131"/>
+      <c r="R7" s="131"/>
+      <c r="S7" s="131"/>
+      <c r="T7" s="131"/>
+      <c r="U7" s="131"/>
+      <c r="V7" s="131"/>
     </row>
     <row r="8" spans="1:36" ht="5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D8" s="7"/>
       <c r="E8" s="6"/>
       <c r="F8" s="30"/>
+      <c r="G8" s="17"/>
+      <c r="H8" s="17"/>
+      <c r="I8" s="33"/>
+      <c r="J8" s="6"/>
+      <c r="K8" s="2"/>
+      <c r="L8" s="2"/>
+      <c r="M8" s="2"/>
+      <c r="N8" s="2"/>
+      <c r="O8" s="2"/>
+      <c r="P8" s="2"/>
+      <c r="Q8" s="2"/>
+      <c r="R8" s="2"/>
+      <c r="S8" s="2"/>
+      <c r="T8" s="2"/>
+      <c r="U8" s="2"/>
+      <c r="V8" s="2"/>
       <c r="W8" s="2"/>
       <c r="X8" s="2"/>
       <c r="Y8" s="2"/>
@@ -2046,6 +2147,26 @@
         <v>8</v>
       </c>
       <c r="F9" s="7"/>
+      <c r="G9" s="130" t="s">
+        <v>71</v>
+      </c>
+      <c r="H9" s="130"/>
+      <c r="I9" s="130"/>
+      <c r="J9" s="131" t="s">
+        <v>72</v>
+      </c>
+      <c r="K9" s="131"/>
+      <c r="L9" s="131"/>
+      <c r="M9" s="2"/>
+      <c r="N9" s="2"/>
+      <c r="O9" s="2"/>
+      <c r="P9" s="2"/>
+      <c r="Q9" s="3"/>
+      <c r="R9" s="2"/>
+      <c r="S9" s="2"/>
+      <c r="T9" s="2"/>
+      <c r="U9" s="3"/>
+      <c r="V9" s="3"/>
       <c r="W9" s="3"/>
       <c r="X9" s="3"/>
       <c r="Y9" s="3"/>
@@ -2055,6 +2176,13 @@
       <c r="D10" s="8"/>
       <c r="E10" s="32"/>
       <c r="F10" s="30"/>
+      <c r="G10" s="17"/>
+      <c r="H10" s="17"/>
+      <c r="I10" s="17"/>
+      <c r="J10" s="30"/>
+      <c r="K10" s="31"/>
+      <c r="L10" s="30"/>
+      <c r="M10" s="13"/>
     </row>
     <row r="11" spans="1:36" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D11" s="5"/>
@@ -2062,11 +2190,29 @@
         <v>9</v>
       </c>
       <c r="F11" s="7"/>
+      <c r="G11" s="130" t="s">
+        <v>10</v>
+      </c>
+      <c r="H11" s="130"/>
+      <c r="I11" s="130"/>
+      <c r="J11" s="131" t="s">
+        <v>73</v>
+      </c>
+      <c r="K11" s="131"/>
+      <c r="L11" s="131"/>
+      <c r="M11" s="12"/>
     </row>
     <row r="12" spans="1:36" ht="5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D12" s="6"/>
       <c r="E12" s="6"/>
       <c r="F12" s="30"/>
+      <c r="G12" s="17"/>
+      <c r="H12" s="17"/>
+      <c r="I12" s="17"/>
+      <c r="J12" s="32"/>
+      <c r="K12" s="12"/>
+      <c r="L12" s="30"/>
+      <c r="M12" s="12"/>
     </row>
     <row r="13" spans="1:36" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D13" s="5"/>
@@ -2074,6 +2220,17 @@
         <v>11</v>
       </c>
       <c r="F13" s="7"/>
+      <c r="G13" s="130" t="s">
+        <v>12</v>
+      </c>
+      <c r="H13" s="130"/>
+      <c r="I13" s="130"/>
+      <c r="J13" s="131" t="s">
+        <v>74</v>
+      </c>
+      <c r="K13" s="131"/>
+      <c r="L13" s="131"/>
+      <c r="M13" s="12"/>
     </row>
     <row r="14" spans="1:36" ht="8" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="C14"/>
@@ -2083,103 +2240,103 @@
       <c r="M14"/>
     </row>
     <row r="15" spans="1:36" s="39" customFormat="1" ht="19.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="102" t="s">
+      <c r="A15" s="91" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="105" t="s">
+      <c r="B15" s="94" t="s">
         <v>14</v>
       </c>
-      <c r="C15" s="106"/>
-      <c r="D15" s="94" t="s">
+      <c r="C15" s="95"/>
+      <c r="D15" s="124" t="s">
         <v>15</v>
       </c>
-      <c r="E15" s="94"/>
-      <c r="F15" s="94"/>
-      <c r="G15" s="94"/>
-      <c r="H15" s="94"/>
-      <c r="I15" s="94"/>
-      <c r="J15" s="94"/>
-      <c r="K15" s="94"/>
-      <c r="L15" s="94"/>
-      <c r="M15" s="95"/>
-      <c r="N15" s="98" t="s">
+      <c r="E15" s="124"/>
+      <c r="F15" s="124"/>
+      <c r="G15" s="124"/>
+      <c r="H15" s="124"/>
+      <c r="I15" s="124"/>
+      <c r="J15" s="124"/>
+      <c r="K15" s="124"/>
+      <c r="L15" s="124"/>
+      <c r="M15" s="125"/>
+      <c r="N15" s="108" t="s">
         <v>16</v>
       </c>
-      <c r="O15" s="91"/>
-      <c r="P15" s="91"/>
-      <c r="Q15" s="91"/>
-      <c r="R15" s="91"/>
-      <c r="S15" s="91"/>
-      <c r="T15" s="91"/>
-      <c r="U15" s="91"/>
-      <c r="V15" s="91"/>
-      <c r="W15" s="92"/>
-      <c r="X15" s="91" t="s">
+      <c r="O15" s="109"/>
+      <c r="P15" s="109"/>
+      <c r="Q15" s="109"/>
+      <c r="R15" s="109"/>
+      <c r="S15" s="109"/>
+      <c r="T15" s="109"/>
+      <c r="U15" s="109"/>
+      <c r="V15" s="109"/>
+      <c r="W15" s="122"/>
+      <c r="X15" s="109" t="s">
         <v>17</v>
       </c>
-      <c r="Y15" s="91"/>
-      <c r="Z15" s="92"/>
-      <c r="AA15" s="120" t="s">
+      <c r="Y15" s="109"/>
+      <c r="Z15" s="122"/>
+      <c r="AA15" s="80" t="s">
         <v>47</v>
       </c>
-      <c r="AB15" s="120"/>
-      <c r="AC15" s="120"/>
-      <c r="AD15" s="121"/>
+      <c r="AB15" s="80"/>
+      <c r="AC15" s="80"/>
+      <c r="AD15" s="81"/>
     </row>
     <row r="16" spans="1:36" s="39" customFormat="1" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="103"/>
-      <c r="B16" s="107"/>
-      <c r="C16" s="108"/>
-      <c r="D16" s="96"/>
-      <c r="E16" s="96"/>
-      <c r="F16" s="96"/>
-      <c r="G16" s="96"/>
-      <c r="H16" s="96"/>
-      <c r="I16" s="96"/>
-      <c r="J16" s="96"/>
-      <c r="K16" s="96"/>
-      <c r="L16" s="96"/>
-      <c r="M16" s="97"/>
-      <c r="N16" s="98" t="s">
+      <c r="A16" s="92"/>
+      <c r="B16" s="96"/>
+      <c r="C16" s="97"/>
+      <c r="D16" s="126"/>
+      <c r="E16" s="126"/>
+      <c r="F16" s="126"/>
+      <c r="G16" s="126"/>
+      <c r="H16" s="126"/>
+      <c r="I16" s="126"/>
+      <c r="J16" s="126"/>
+      <c r="K16" s="126"/>
+      <c r="L16" s="126"/>
+      <c r="M16" s="127"/>
+      <c r="N16" s="108" t="s">
         <v>18</v>
       </c>
-      <c r="O16" s="91"/>
-      <c r="P16" s="91"/>
-      <c r="Q16" s="118"/>
-      <c r="R16" s="98" t="s">
+      <c r="O16" s="109"/>
+      <c r="P16" s="109"/>
+      <c r="Q16" s="110"/>
+      <c r="R16" s="108" t="s">
         <v>19</v>
       </c>
-      <c r="S16" s="91"/>
-      <c r="T16" s="91"/>
-      <c r="U16" s="118"/>
-      <c r="V16" s="116" t="s">
+      <c r="S16" s="109"/>
+      <c r="T16" s="109"/>
+      <c r="U16" s="110"/>
+      <c r="V16" s="106" t="s">
         <v>20</v>
       </c>
-      <c r="W16" s="109" t="s">
+      <c r="W16" s="98" t="s">
         <v>55</v>
       </c>
-      <c r="X16" s="87" t="s">
+      <c r="X16" s="118" t="s">
         <v>49</v>
       </c>
-      <c r="Y16" s="89" t="s">
+      <c r="Y16" s="120" t="s">
         <v>45</v>
       </c>
-      <c r="Z16" s="126" t="s">
+      <c r="Z16" s="86" t="s">
         <v>46</v>
       </c>
-      <c r="AA16" s="122" t="s">
+      <c r="AA16" s="82" t="s">
         <v>54</v>
       </c>
-      <c r="AB16" s="123"/>
-      <c r="AC16" s="124" t="s">
+      <c r="AB16" s="83"/>
+      <c r="AC16" s="84" t="s">
         <v>50</v>
       </c>
-      <c r="AD16" s="124" t="s">
+      <c r="AD16" s="84" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="17" spans="1:30" s="44" customFormat="1" ht="44" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="104"/>
+      <c r="A17" s="93"/>
       <c r="B17" s="41" t="s">
         <v>21</v>
       </c>
@@ -2240,19 +2397,19 @@
       <c r="U17" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="V17" s="117"/>
-      <c r="W17" s="110"/>
-      <c r="X17" s="88"/>
-      <c r="Y17" s="90"/>
-      <c r="Z17" s="127"/>
+      <c r="V17" s="107"/>
+      <c r="W17" s="99"/>
+      <c r="X17" s="119"/>
+      <c r="Y17" s="121"/>
+      <c r="Z17" s="87"/>
       <c r="AA17" s="49" t="s">
         <v>52</v>
       </c>
       <c r="AB17" s="38" t="s">
         <v>53</v>
       </c>
-      <c r="AC17" s="125"/>
-      <c r="AD17" s="125"/>
+      <c r="AC17" s="85"/>
+      <c r="AD17" s="85"/>
     </row>
     <row r="18" spans="1:30" ht="44" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A18" s="18" t="s">
@@ -2293,19 +2450,19 @@
       <c r="AD18" s="47"/>
     </row>
     <row r="19" spans="1:30" ht="44" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="93" t="s">
+      <c r="A19" s="123" t="s">
         <v>66</v>
       </c>
-      <c r="B19" s="93"/>
-      <c r="C19" s="93"/>
-      <c r="D19" s="93"/>
-      <c r="E19" s="93"/>
+      <c r="B19" s="123"/>
+      <c r="C19" s="123"/>
+      <c r="D19" s="123"/>
+      <c r="E19" s="123"/>
       <c r="F19" s="36"/>
       <c r="H19" s="11"/>
-      <c r="L19" s="115" t="s">
+      <c r="L19" s="104" t="s">
         <v>42</v>
       </c>
-      <c r="M19" s="115"/>
+      <c r="M19" s="104"/>
       <c r="N19" s="64"/>
       <c r="O19" s="65"/>
       <c r="P19" s="66"/>
@@ -2325,69 +2482,69 @@
       <c r="AD19" s="47"/>
     </row>
     <row r="20" spans="1:30" ht="75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="111" t="s">
+      <c r="A20" s="100" t="s">
         <v>56</v>
       </c>
-      <c r="B20" s="111"/>
-      <c r="C20" s="111"/>
-      <c r="D20" s="111"/>
-      <c r="E20" s="111"/>
+      <c r="B20" s="100"/>
+      <c r="C20" s="100"/>
+      <c r="D20" s="100"/>
+      <c r="E20" s="100"/>
       <c r="H20" s="11"/>
-      <c r="L20" s="86" t="s">
+      <c r="L20" s="105" t="s">
         <v>43</v>
       </c>
-      <c r="M20" s="86"/>
-      <c r="N20" s="112"/>
-      <c r="O20" s="113"/>
-      <c r="P20" s="113"/>
-      <c r="Q20" s="113"/>
-      <c r="R20" s="113"/>
-      <c r="S20" s="113"/>
-      <c r="T20" s="113"/>
-      <c r="U20" s="113"/>
-      <c r="V20" s="114"/>
+      <c r="M20" s="105"/>
+      <c r="N20" s="101"/>
+      <c r="O20" s="102"/>
+      <c r="P20" s="102"/>
+      <c r="Q20" s="102"/>
+      <c r="R20" s="102"/>
+      <c r="S20" s="102"/>
+      <c r="T20" s="102"/>
+      <c r="U20" s="102"/>
+      <c r="V20" s="103"/>
       <c r="W20" s="67"/>
     </row>
     <row r="21" spans="1:30" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="119" t="s">
+      <c r="A21" s="111" t="s">
         <v>67</v>
       </c>
-      <c r="B21" s="119"/>
-      <c r="C21" s="119"/>
-      <c r="D21" s="119"/>
-      <c r="E21" s="119"/>
+      <c r="B21" s="111"/>
+      <c r="C21" s="111"/>
+      <c r="D21" s="111"/>
+      <c r="E21" s="111"/>
       <c r="H21" s="11"/>
-      <c r="L21" s="86" t="s">
+      <c r="L21" s="105" t="s">
         <v>40</v>
       </c>
-      <c r="M21" s="86"/>
-      <c r="N21" s="99"/>
-      <c r="O21" s="100"/>
-      <c r="P21" s="100"/>
-      <c r="Q21" s="100"/>
-      <c r="R21" s="100"/>
-      <c r="S21" s="100"/>
-      <c r="T21" s="100"/>
-      <c r="U21" s="100"/>
-      <c r="V21" s="100"/>
-      <c r="W21" s="101"/>
+      <c r="M21" s="105"/>
+      <c r="N21" s="88"/>
+      <c r="O21" s="89"/>
+      <c r="P21" s="89"/>
+      <c r="Q21" s="89"/>
+      <c r="R21" s="89"/>
+      <c r="S21" s="89"/>
+      <c r="T21" s="89"/>
+      <c r="U21" s="89"/>
+      <c r="V21" s="89"/>
+      <c r="W21" s="90"/>
     </row>
     <row r="22" spans="1:30" ht="31" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A22" s="4"/>
       <c r="H22" s="11"/>
-      <c r="L22" s="86" t="s">
+      <c r="L22" s="105" t="s">
         <v>57</v>
       </c>
-      <c r="M22" s="86"/>
-      <c r="N22" s="99"/>
-      <c r="O22" s="100"/>
-      <c r="P22" s="100"/>
-      <c r="Q22" s="100"/>
-      <c r="R22" s="100"/>
-      <c r="S22" s="100"/>
-      <c r="T22" s="100"/>
-      <c r="U22" s="100"/>
-      <c r="V22" s="101"/>
+      <c r="M22" s="105"/>
+      <c r="N22" s="88"/>
+      <c r="O22" s="89"/>
+      <c r="P22" s="89"/>
+      <c r="Q22" s="89"/>
+      <c r="R22" s="89"/>
+      <c r="S22" s="89"/>
+      <c r="T22" s="89"/>
+      <c r="U22" s="89"/>
+      <c r="V22" s="90"/>
       <c r="W22" s="67"/>
     </row>
     <row r="23" spans="1:30" ht="16" thickBot="1" x14ac:dyDescent="0.25">
@@ -2404,9 +2561,9 @@
       <c r="AA24" s="61" t="s">
         <v>37</v>
       </c>
-      <c r="AB24" s="81"/>
-      <c r="AC24" s="82"/>
-      <c r="AD24" s="83"/>
+      <c r="AB24" s="113"/>
+      <c r="AC24" s="114"/>
+      <c r="AD24" s="115"/>
     </row>
     <row r="25" spans="1:30" ht="34" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A25" s="11"/>
@@ -2420,39 +2577,31 @@
       <c r="AA25" s="61" t="s">
         <v>39</v>
       </c>
-      <c r="AB25" s="81"/>
-      <c r="AC25" s="82"/>
-      <c r="AD25" s="83"/>
+      <c r="AB25" s="113"/>
+      <c r="AC25" s="114"/>
+      <c r="AD25" s="115"/>
     </row>
     <row r="27" spans="1:30" ht="111" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="80" t="s">
+      <c r="A27" s="112" t="s">
         <v>64</v>
       </c>
-      <c r="B27" s="80"/>
-      <c r="C27" s="80"/>
-      <c r="D27" s="80"/>
-      <c r="E27" s="80"/>
+      <c r="B27" s="112"/>
+      <c r="C27" s="112"/>
+      <c r="D27" s="112"/>
+      <c r="E27" s="112"/>
     </row>
   </sheetData>
-  <mergeCells count="32">
-    <mergeCell ref="AA15:AD15"/>
-    <mergeCell ref="AA16:AB16"/>
-    <mergeCell ref="AC16:AC17"/>
-    <mergeCell ref="AD16:AD17"/>
-    <mergeCell ref="Z16:Z17"/>
-    <mergeCell ref="N22:V22"/>
-    <mergeCell ref="A15:A17"/>
-    <mergeCell ref="B15:C16"/>
-    <mergeCell ref="W16:W17"/>
-    <mergeCell ref="A20:E20"/>
-    <mergeCell ref="N20:V20"/>
-    <mergeCell ref="N21:W21"/>
-    <mergeCell ref="L19:M19"/>
-    <mergeCell ref="L20:M20"/>
-    <mergeCell ref="V16:V17"/>
-    <mergeCell ref="R16:U16"/>
-    <mergeCell ref="N16:Q16"/>
-    <mergeCell ref="A21:E21"/>
+  <mergeCells count="44">
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="J11:L11"/>
+    <mergeCell ref="G13:I13"/>
+    <mergeCell ref="J13:L13"/>
+    <mergeCell ref="G6:I6"/>
+    <mergeCell ref="J6:V6"/>
+    <mergeCell ref="G7:I7"/>
+    <mergeCell ref="J7:V7"/>
+    <mergeCell ref="G9:I9"/>
+    <mergeCell ref="J9:L9"/>
     <mergeCell ref="A27:E27"/>
     <mergeCell ref="AB25:AD25"/>
     <mergeCell ref="A1:AD1"/>
@@ -2467,6 +2616,26 @@
     <mergeCell ref="L21:M21"/>
     <mergeCell ref="D15:M16"/>
     <mergeCell ref="N15:W15"/>
+    <mergeCell ref="G5:I5"/>
+    <mergeCell ref="J5:L5"/>
+    <mergeCell ref="N22:V22"/>
+    <mergeCell ref="A15:A17"/>
+    <mergeCell ref="B15:C16"/>
+    <mergeCell ref="W16:W17"/>
+    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="N20:V20"/>
+    <mergeCell ref="N21:W21"/>
+    <mergeCell ref="L19:M19"/>
+    <mergeCell ref="L20:M20"/>
+    <mergeCell ref="V16:V17"/>
+    <mergeCell ref="R16:U16"/>
+    <mergeCell ref="N16:Q16"/>
+    <mergeCell ref="A21:E21"/>
+    <mergeCell ref="AA15:AD15"/>
+    <mergeCell ref="AA16:AB16"/>
+    <mergeCell ref="AC16:AC17"/>
+    <mergeCell ref="AD16:AD17"/>
+    <mergeCell ref="Z16:Z17"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -2871,15 +3040,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000B7BBE98651F7A43AC7BF2F06836443C" ma:contentTypeVersion="12" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="b51c7281b06024c9ff887df9fe3bb465">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="8103b6e4-b1cc-417b-af38-f980b3f4bdef" xmlns:ns3="026a8ae5-d6a9-4af7-bf98-fe61cc11d283" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c056a6abdadb071051b2c083c327215c" ns2:_="" ns3:_="">
     <xsd:import namespace="8103b6e4-b1cc-417b-af38-f980b3f4bdef"/>
@@ -3096,6 +3256,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DE9C2EEE-EA72-4039-9998-752A033046FC}">
   <ds:schemaRefs>
@@ -3108,14 +3277,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AD87B94F-381C-458D-A5C9-64DD7F51B7FF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E02BC65-B354-4988-8893-F98AC7F212AA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3132,4 +3293,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AD87B94F-381C-458D-A5C9-64DD7F51B7FF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>